<commit_message>
QLDA: fix(ke-hoach-trien-khai-hang-muc): nâng cấp import Excel template và luồng import.
Cho phép import chỉ với file; map dự án và buocId tùy chọn. Giai đoạn theo quy trình dự án, combo đơn vị/cán bộ phối hợp nhiều giá trị.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/QLDA.WebApi/PrintTemplates/Import_KeHoachTrienKhaiHangMuc.xlsx
+++ b/QLDA.WebApi/PrintTemplates/Import_KeHoachTrienKhaiHangMuc.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\SER\QLDA.WebApi\PrintTemplates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37EE631A-9448-4BA3-950F-27F5D0EA6F49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7422DEAC-C08D-462C-A777-846D967FF88C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="26">
   <si>
     <t>ỦY BAN NHÂN DÂN THÀNH PHỐ HỒ CHÍ MINH
 TRUNG TÂM CHUYỂN ĐỔI SỐ</t>
@@ -35,7 +35,7 @@
     <t>MẪU IMPORT KẾ HOẠCH TRIỂN KHAI HẠNG MỤC</t>
   </si>
   <si>
-    <t>Nhập dữ liệu vào bảng bên dưới. Dự án / Giai đoạn / Đơn vị / Cán bộ chọn từ danh sách. Đơn vị phối hợp và Cán bộ phối hợp: nhập nhiều giá trị, cách nhau dấu phẩy. Ngày nhập dd/MM/yyyy.</t>
+    <t>Nhập dữ liệu vào bảng bên dưới. Dự án / Giai đoạn / Đơn vị / Cán bộ chọn từ danh sách. Đơn vị phối hợp và Cán bộ phối hợp: chọn từ danh sách, nhiều giá trị cách nhau dấu phẩy (vd: Phòng A, Phòng B). Ngày nhập dd/MM/yyyy.</t>
   </si>
   <si>
     <t>Dự án</t>
@@ -80,9 +80,6 @@
     <t>Chọn từ danh mục</t>
   </si>
   <si>
-    <t>Tùy chọn — nhiều giá trị, cách nhau dấu phẩy</t>
-  </si>
-  <si>
     <t>dd/MM/yyyy</t>
   </si>
   <si>
@@ -98,7 +95,13 @@
     <t>$cbo3</t>
   </si>
   <si>
+    <t>$cbo5</t>
+  </si>
+  <si>
     <t>$cbo4</t>
+  </si>
+  <si>
+    <t>$cbo6</t>
   </si>
 </sst>
 </file>
@@ -108,7 +111,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
   </numFmts>
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -147,19 +150,6 @@
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Times New Roman"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="Times New Roman"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -208,7 +198,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyBorder="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -219,6 +209,15 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
@@ -238,33 +237,11 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Bình thường" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="1">
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="3"/>
-      </font>
-    </dxf>
-  </dxfs>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -278,7 +255,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="KeHoachTrienKhaiHangMucImport" displayName="KeHoachTrienKhaiHangMucImport" ref="A5:K7" totalsRowShown="0" headerRowDxfId="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="KeHoachTrienKhaiHangMucImport" displayName="KeHoachTrienKhaiHangMucImport" ref="A5:K7" totalsRowShown="0">
   <tableColumns count="11">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Dự án"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Tên hạng mục"/>
@@ -324,9 +301,27 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="Combo4" displayName="Combo4" ref="F1:F2" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="Combo5" displayName="Combo5" ref="E1:E2" totalsRowShown="0">
   <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0400-000001000000}" name="$cbo4"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0400-000001000000}" name="$cbo5"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{00000000-000C-0000-FFFF-FFFF05000000}" name="Combo4" displayName="Combo4" ref="F1:F2" totalsRowShown="0">
+  <tableColumns count="1">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0500-000001000000}" name="$cbo4"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{00000000-000C-0000-FFFF-FFFF06000000}" name="Combo6" displayName="Combo6" ref="G1:G2" totalsRowShown="0">
+  <tableColumns count="1">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0600-000001000000}" name="$cbo6"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -691,96 +686,100 @@
       <c r="J4" s="1"/>
       <c r="K4" s="1"/>
     </row>
-    <row r="5" spans="1:11" s="14" customFormat="1" ht="28.2" x14ac:dyDescent="0.3">
-      <c r="A5" s="11" t="s">
+    <row r="5" spans="1:11" ht="28.2" x14ac:dyDescent="0.3">
+      <c r="A5" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="11" t="s">
+      <c r="B5" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="11" t="s">
+      <c r="C5" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="D5" s="11" t="s">
+      <c r="D5" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="E5" s="11" t="s">
+      <c r="E5" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="F5" s="11" t="s">
+      <c r="F5" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="G5" s="11" t="s">
+      <c r="G5" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="H5" s="12" t="s">
+      <c r="H5" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="I5" s="12" t="s">
+      <c r="I5" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="J5" s="13" t="s">
+      <c r="J5" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="K5" s="12" t="s">
+      <c r="K5" s="5" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="28.2" x14ac:dyDescent="0.3">
-      <c r="A6" s="4" t="s">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A6" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C6" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="D6" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="E6" s="5" t="s">
+      <c r="E6" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="G6" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="H6" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="F6" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="G6" s="5" t="s">
+      <c r="I6" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="H6" s="5" t="s">
+      <c r="J6" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="I6" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="J6" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="K6" s="5" t="s">
-        <v>19</v>
+      <c r="K6" s="8" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A7" s="6" t="s">
+      <c r="A7" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="B7" s="9"/>
+      <c r="C7" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="B7" s="6"/>
-      <c r="C7" s="7" t="s">
+      <c r="D7" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="D7" s="6" t="s">
+      <c r="E7" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="E7" s="6"/>
-      <c r="F7" s="6" t="s">
+      <c r="F7" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="G7" s="6"/>
-      <c r="H7" s="8"/>
-      <c r="I7" s="8"/>
-      <c r="J7" s="9"/>
-      <c r="K7" s="8"/>
+      <c r="G7" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="H7" s="11"/>
+      <c r="I7" s="11"/>
+      <c r="J7" s="12"/>
+      <c r="K7" s="11"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -798,30 +797,38 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:G1"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A1" s="10" t="s">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A1" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="C1" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="C1" s="10" t="s">
+      <c r="D1" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="D1" s="10" t="s">
+      <c r="E1" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="F1" s="10" t="s">
+      <c r="F1" s="13" t="s">
         <v>24</v>
+      </c>
+      <c r="G1" s="13" t="s">
+        <v>25</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
-  <tableParts count="4">
+  <tableParts count="6">
     <tablePart r:id="rId1"/>
     <tablePart r:id="rId2"/>
     <tablePart r:id="rId3"/>
     <tablePart r:id="rId4"/>
+    <tablePart r:id="rId5"/>
+    <tablePart r:id="rId6"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>